<commit_message>
cambio de colores, filtros, highligts
</commit_message>
<xml_diff>
--- a/data/roles_areas.xlsx
+++ b/data/roles_areas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Inventario\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F58EBE-1CCE-4B81-BFCA-60B703E8BD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0C1D12-9498-435B-9D13-65DE65B05CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8F2D9A4D-AB14-4069-820F-8029A79ED844}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F2D9A4D-AB14-4069-820F-8029A79ED844}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5349,12 +5349,12 @@
   <dimension ref="A1:F1537"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>